<commit_message>
Neutralité : exemples d'EID neutres, modèles Excel sans données réelles, listes de départ vides, allowBackup=false
- Exemples de saisie : ex: 250 000000 000000 (4 champs d'EID), ex: 000000 pour l'indicatif de marquage.
- Modèles Excel d'import (embarqués et copies de tests/fixtures/modeles) : EID d'exemple neutres
  (mêmes 5 derniers chiffres, les cas de doublon restent des doublons), n° SIEOL d'exemple du
  contrôle laitier neutres, nom de personne retiré des métadonnées, en-tête « 11 ou 15 chiffres »
  pour Nouveaux animaux.
- Compte neuf : vaccins et antiparasitaires vides, aucun prix de référence négocié (l'entrée 2025
  n'est créée que pour un compte qui a déjà des données de lait).
- AndroidManifest : allowBackup=false.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLuVdepQJH57EG96mn2Beh
</commit_message>
<xml_diff>
--- a/tests/fixtures/modeles/Modele_Controle_Laitier.xlsx
+++ b/tests/fixtures/modeles/Modele_Controle_Laitier.xlsx
@@ -57,7 +57,7 @@
     <t>Contrôle 3 (mL[/code])</t>
   </si>
   <si>
-    <t>180055</t>
+    <t>250101</t>
   </si>
   <si>
     <t>1440</t>
@@ -69,7 +69,7 @@
     <t>1060</t>
   </si>
   <si>
-    <t>180133</t>
+    <t>250102</t>
   </si>
   <si>
     <t>1620/01</t>
@@ -81,7 +81,7 @@
     <t>840</t>
   </si>
   <si>
-    <t>190059</t>
+    <t>250103</t>
   </si>
   <si>
     <t>09</t>
@@ -90,7 +90,7 @@
     <t>1200</t>
   </si>
   <si>
-    <t>190069</t>
+    <t>250104</t>
   </si>
   <si>
     <t>07</t>
@@ -102,7 +102,7 @@
     <t>900</t>
   </si>
   <si>
-    <t>190085</t>
+    <t>250105</t>
   </si>
   <si>
     <t>1460/08</t>

</xml_diff>